<commit_message>
fix(tora): AUTEF preservado no add/update (tabela.js) + coluna AUTEF na impressao
</commit_message>
<xml_diff>
--- a/assets/modelos/Modelo_Romaneio_Tora_import.xlsx
+++ b/assets/modelos/Modelo_Romaneio_Tora_import.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sisweb\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Sisweb\assets\modelos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2234670-63EA-4D1E-B16B-CF4545132FCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61B5AB2E-C687-41D0-886F-A5ADAEB607B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{EAA124F4-DE81-479E-B9CF-6598A60B4081}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="41">
   <si>
     <t>Plaqueta</t>
   </si>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t>X4</t>
-  </si>
-  <si>
-    <t>V. Geo.</t>
   </si>
   <si>
     <t>Valor</t>
@@ -588,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18CEAF4E-6327-4E91-8BF8-6A5325A23B0E}">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -599,11 +596,11 @@
     <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.88671875" customWidth="1"/>
     <col min="8" max="8" width="9.44140625" customWidth="1"/>
-    <col min="9" max="14" width="9.33203125" customWidth="1"/>
-    <col min="15" max="16" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="13" width="9.33203125" customWidth="1"/>
+    <col min="14" max="15" width="10.5546875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -643,28 +640,25 @@
       <c r="M1" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>200</v>
@@ -693,22 +687,22 @@
       <c r="M2">
         <v>65</v>
       </c>
-      <c r="O2" s="2">
+      <c r="N2" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3">
         <v>160</v>
@@ -737,22 +731,22 @@
       <c r="M3">
         <v>46</v>
       </c>
-      <c r="O3" s="2">
+      <c r="N3" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E4">
         <v>160</v>
@@ -781,22 +775,22 @@
       <c r="M4">
         <v>46</v>
       </c>
-      <c r="O4" s="2">
+      <c r="N4" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E5">
         <v>156</v>
@@ -825,22 +819,22 @@
       <c r="M5">
         <v>40</v>
       </c>
-      <c r="O5" s="2">
+      <c r="N5" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E6">
         <v>166</v>
@@ -869,22 +863,22 @@
       <c r="M6">
         <v>46</v>
       </c>
-      <c r="O6" s="2">
+      <c r="N6" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="E7">
         <v>170</v>
@@ -913,22 +907,22 @@
       <c r="M7">
         <v>48</v>
       </c>
-      <c r="O7" s="2">
+      <c r="N7" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E8">
         <v>150</v>
@@ -957,22 +951,22 @@
       <c r="M8">
         <v>54</v>
       </c>
-      <c r="O8" s="2">
+      <c r="N8" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9">
         <v>172</v>
@@ -1001,22 +995,22 @@
       <c r="M9">
         <v>48</v>
       </c>
-      <c r="O9" s="2">
+      <c r="N9" s="2">
         <v>650</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
       <c r="D10" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E10">
         <v>230</v>
@@ -1045,7 +1039,7 @@
       <c r="M10">
         <v>72</v>
       </c>
-      <c r="O10" s="2">
+      <c r="N10" s="2">
         <v>650</v>
       </c>
     </row>

</xml_diff>